<commit_message>
Added new Selenium scripts and updated existing codes
</commit_message>
<xml_diff>
--- a/src/test/java/testdata/LoginData.xlsx
+++ b/src/test/java/testdata/LoginData.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Work_Samples\OrangeHRMAutomation\src\test\java\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2C49B2C-C8C9-44E2-8CA5-A1612386AD64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{147D58F2-82B5-454F-9A1B-B7C7B02BAE5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LOGIN_PAGE" sheetId="1" r:id="rId1"/>
+    <sheet name="ADD EMPLOYEE" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>Admin</t>
   </si>
@@ -37,6 +38,24 @@
   </si>
   <si>
     <t>Password</t>
+  </si>
+  <si>
+    <t>Firstname</t>
+  </si>
+  <si>
+    <t>Lastname</t>
+  </si>
+  <si>
+    <t>Middlename</t>
+  </si>
+  <si>
+    <t>Mihir</t>
+  </si>
+  <si>
+    <t>Ranjan</t>
+  </si>
+  <si>
+    <t>Panda</t>
   </si>
 </sst>
 </file>
@@ -381,4 +400,39 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18E657C6-3BD5-4CA0-A209-E3B334C36EE5}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="3" width="11.81640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>